<commit_message>
fix(gt): blank Value column in metadata template so Judah samples stop leaking
The metadata sheet in _template.xlsx pre-filled every field with Judah-flavored
sample values ("judah-vs-ofc-2026-04-25", "OFC 2016", "black", etc.) in column
B (Value). Coaches copying the template for a new match had to remember to
overwrite each cell — anything they missed shipped through to eval JSON as if
it were real ground truth.

Value column now starts blank; sample format moved into Notes column as "e.g. …"
so users still see guidance without the trap. Regenerated _template.xlsx and
added Fusion 2008 (2015-11-20 tentative date) GT with only Joshua's provided
fields populated.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/scripts/ground-truth/_template.xlsx
+++ b/scripts/ground-truth/_template.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="158" uniqueCount="110">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="168" uniqueCount="108">
   <si>
     <t>STIX Match Ground-Truth Tagger</t>
   </si>
@@ -122,79 +122,73 @@
     <t>Match name</t>
   </si>
   <si>
-    <t>judah-vs-ofc-2026-04-25</t>
-  </si>
-  <si>
-    <t>Short slug for the match (used as filename and id)</t>
+    <t>Short slug for the match (used as filename and id) — e.g. judah-vs-ofc-2026-04-25</t>
   </si>
   <si>
     <t>Date</t>
   </si>
   <si>
-    <t>2026-04-25</t>
-  </si>
-  <si>
-    <t>YYYY-MM-DD</t>
+    <t>YYYY-MM-DD — e.g. 2026-04-25</t>
   </si>
   <si>
     <t>Opponent</t>
   </si>
   <si>
-    <t>OFC 2016</t>
-  </si>
-  <si>
-    <t>Opposition team name</t>
+    <t>Opposition team name — e.g. OFC 2016</t>
   </si>
   <si>
     <t>Venue</t>
   </si>
   <si>
-    <t>Home</t>
+    <t>e.g. Home</t>
   </si>
   <si>
     <t>Session type</t>
   </si>
   <si>
-    <t>Match</t>
+    <t>e.g. Match</t>
   </si>
   <si>
     <t>My team color</t>
   </si>
   <si>
-    <t>black</t>
-  </si>
-  <si>
-    <t>Outfield jersey colour, lowercase</t>
+    <t>Outfield jersey colour, lowercase — e.g. black</t>
   </si>
   <si>
     <t>Opponent color</t>
   </si>
   <si>
-    <t>light blue</t>
+    <t>e.g. light blue</t>
   </si>
   <si>
     <t>My GK color</t>
   </si>
   <si>
-    <t>orange</t>
+    <t>e.g. orange</t>
   </si>
   <si>
     <t>Age group</t>
   </si>
   <si>
-    <t>U10</t>
+    <t>e.g. U10</t>
   </si>
   <si>
     <t>Video duration (MM:SS)</t>
   </si>
   <si>
-    <t>52:23</t>
+    <t>e.g. 52:23</t>
   </si>
   <si>
     <t>Final score — us</t>
   </si>
   <si>
+    <t>e.g. 4</t>
+  </si>
+  <si>
     <t>Final score — them</t>
+  </si>
+  <si>
+    <t>e.g. 1</t>
   </si>
   <si>
     <t>Us GK sub at (MM:SS)</t>
@@ -978,140 +972,164 @@
         <v>33</v>
       </c>
       <c r="B2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2" t="s">
         <v>34</v>
-      </c>
-      <c r="C2" t="s">
-        <v>35</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>35</v>
+      </c>
+      <c r="B3" t="s">
+        <v>1</v>
+      </c>
+      <c r="C3" t="s">
         <v>36</v>
-      </c>
-      <c r="B3" t="s">
-        <v>37</v>
-      </c>
-      <c r="C3" t="s">
-        <v>38</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
+        <v>37</v>
+      </c>
+      <c r="B4" t="s">
+        <v>1</v>
+      </c>
+      <c r="C4" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
         <v>39</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B5" t="s">
+        <v>1</v>
+      </c>
+      <c r="C5" t="s">
         <v>40</v>
       </c>
-      <c r="C4" t="s">
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
         <v>41</v>
       </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
+      <c r="B6" t="s">
+        <v>1</v>
+      </c>
+      <c r="C6" t="s">
         <v>42</v>
-      </c>
-      <c r="B5" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>44</v>
-      </c>
-      <c r="B6" t="s">
-        <v>45</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
+        <v>43</v>
+      </c>
+      <c r="B7" t="s">
+        <v>1</v>
+      </c>
+      <c r="C7" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>45</v>
+      </c>
+      <c r="B8" t="s">
+        <v>1</v>
+      </c>
+      <c r="C8" t="s">
         <v>46</v>
       </c>
-      <c r="B7" t="s">
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
         <v>47</v>
       </c>
-      <c r="C7" t="s">
+      <c r="B9" t="s">
+        <v>1</v>
+      </c>
+      <c r="C9" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
         <v>49</v>
       </c>
-      <c r="B8" t="s">
+      <c r="B10" t="s">
+        <v>1</v>
+      </c>
+      <c r="C10" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
         <v>51</v>
       </c>
-      <c r="B9" t="s">
+      <c r="B11" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="C11" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
         <v>53</v>
       </c>
-      <c r="B10" t="s">
+      <c r="B12" t="s">
+        <v>1</v>
+      </c>
+      <c r="C12" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
         <v>55</v>
       </c>
-      <c r="B11" s="5" t="s">
+      <c r="B13" t="s">
+        <v>1</v>
+      </c>
+      <c r="C13" t="s">
         <v>56</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
-        <v>57</v>
-      </c>
-      <c r="B12">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
-        <v>58</v>
-      </c>
-      <c r="B13">
-        <v>1</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="B14" s="5" t="s">
         <v>1</v>
       </c>
       <c r="C14" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="B15" s="5" t="s">
         <v>1</v>
       </c>
       <c r="C15" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="B16" t="s">
         <v>1</v>
       </c>
       <c r="C16" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
     </row>
   </sheetData>
@@ -1151,37 +1169,37 @@
   <sheetData>
     <row r="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="C1" s="4" t="s">
         <v>65</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="D1" s="4" t="s">
         <v>66</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="E1" s="4" t="s">
         <v>67</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="F1" s="4" t="s">
         <v>68</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="G1" s="4" t="s">
         <v>69</v>
       </c>
-      <c r="F1" s="4" t="s">
+      <c r="H1" s="4" t="s">
         <v>70</v>
       </c>
-      <c r="G1" s="4" t="s">
+      <c r="I1" s="4" t="s">
         <v>71</v>
       </c>
-      <c r="H1" s="4" t="s">
+      <c r="J1" s="4" t="s">
         <v>72</v>
       </c>
-      <c r="I1" s="4" t="s">
+      <c r="K1" s="4" t="s">
         <v>73</v>
-      </c>
-      <c r="J1" s="4" t="s">
-        <v>74</v>
-      </c>
-      <c r="K1" s="4" t="s">
-        <v>75</v>
       </c>
       <c r="L1" s="4" t="s">
         <v>32</v>
@@ -1864,46 +1882,46 @@
   <sheetData>
     <row r="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="C1" s="4" t="s">
         <v>65</v>
       </c>
-      <c r="B1" s="4" t="s">
-        <v>66</v>
-      </c>
-      <c r="C1" s="4" t="s">
-        <v>67</v>
-      </c>
       <c r="D1" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="E1" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="F1" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="G1" s="4" t="s">
         <v>76</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="H1" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="I1" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="J1" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="K1" s="4" t="s">
         <v>70</v>
       </c>
-      <c r="F1" s="4" t="s">
-        <v>77</v>
-      </c>
-      <c r="G1" s="4" t="s">
-        <v>78</v>
-      </c>
-      <c r="H1" s="4" t="s">
-        <v>79</v>
-      </c>
-      <c r="I1" s="4" t="s">
-        <v>80</v>
-      </c>
-      <c r="J1" s="4" t="s">
-        <v>81</v>
-      </c>
-      <c r="K1" s="4" t="s">
+      <c r="L1" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="M1" s="4" t="s">
         <v>72</v>
       </c>
-      <c r="L1" s="4" t="s">
+      <c r="N1" s="4" t="s">
         <v>73</v>
-      </c>
-      <c r="M1" s="4" t="s">
-        <v>74</v>
-      </c>
-      <c r="N1" s="4" t="s">
-        <v>75</v>
       </c>
       <c r="O1" s="4" t="s">
         <v>32</v>
@@ -2610,7 +2628,7 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="B1" s="6"/>
       <c r="C1" s="6"/>
@@ -2620,7 +2638,7 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="B2" s="6"/>
       <c r="C2" s="6"/>
@@ -2630,7 +2648,7 @@
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="B4" t="s">
         <v>1</v>
@@ -2638,7 +2656,7 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="B5" t="s">
         <v>1</v>
@@ -2646,7 +2664,7 @@
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="B6" t="s">
         <v>1</v>
@@ -2654,7 +2672,7 @@
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="B7" t="s">
         <v>1</v>
@@ -2662,7 +2680,7 @@
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="B8" t="s">
         <v>1</v>
@@ -2670,7 +2688,7 @@
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="B9" t="s">
         <v>1</v>
@@ -2678,7 +2696,7 @@
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="B10" t="s">
         <v>1</v>
@@ -2686,7 +2704,7 @@
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="B11" t="s">
         <v>1</v>
@@ -2694,7 +2712,7 @@
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="B12" t="s">
         <v>1</v>
@@ -2702,7 +2720,7 @@
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="B13" t="s">
         <v>1</v>
@@ -2710,37 +2728,37 @@
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A16" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="B16" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="C16" s="4" t="s">
         <v>65</v>
       </c>
-      <c r="B16" s="4" t="s">
-        <v>66</v>
-      </c>
-      <c r="C16" s="4" t="s">
-        <v>67</v>
-      </c>
       <c r="D16" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="E16" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="F16" s="4" t="s">
         <v>94</v>
       </c>
-      <c r="E16" s="4" t="s">
+      <c r="G16" s="4" t="s">
         <v>95</v>
       </c>
-      <c r="F16" s="4" t="s">
+      <c r="H16" s="4" t="s">
         <v>96</v>
       </c>
-      <c r="G16" s="4" t="s">
+      <c r="I16" s="4" t="s">
         <v>97</v>
       </c>
-      <c r="H16" s="4" t="s">
+      <c r="J16" s="4" t="s">
         <v>98</v>
       </c>
-      <c r="I16" s="4" t="s">
+      <c r="K16" s="4" t="s">
         <v>99</v>
-      </c>
-      <c r="J16" s="4" t="s">
-        <v>100</v>
-      </c>
-      <c r="K16" s="4" t="s">
-        <v>101</v>
       </c>
       <c r="L16" s="4" t="s">
         <v>32</v>
@@ -3434,31 +3452,31 @@
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="C1" s="4" t="s">
         <v>65</v>
       </c>
-      <c r="B1" s="4" t="s">
-        <v>66</v>
-      </c>
-      <c r="C1" s="4" t="s">
-        <v>67</v>
-      </c>
       <c r="D1" s="4" t="s">
+        <v>100</v>
+      </c>
+      <c r="E1" s="4" t="s">
+        <v>101</v>
+      </c>
+      <c r="F1" s="4" t="s">
         <v>102</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="G1" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="H1" s="4" t="s">
         <v>103</v>
       </c>
-      <c r="F1" s="4" t="s">
-        <v>104</v>
-      </c>
-      <c r="G1" s="4" t="s">
+      <c r="I1" s="4" t="s">
         <v>78</v>
-      </c>
-      <c r="H1" s="4" t="s">
-        <v>105</v>
-      </c>
-      <c r="I1" s="4" t="s">
-        <v>80</v>
       </c>
       <c r="J1" s="4" t="s">
         <v>32</v>
@@ -4143,28 +4161,28 @@
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="C1" s="4" t="s">
         <v>65</v>
       </c>
-      <c r="B1" s="4" t="s">
-        <v>66</v>
-      </c>
-      <c r="C1" s="4" t="s">
-        <v>67</v>
-      </c>
       <c r="D1" s="4" t="s">
+        <v>104</v>
+      </c>
+      <c r="E1" s="4" t="s">
+        <v>105</v>
+      </c>
+      <c r="F1" s="4" t="s">
+        <v>94</v>
+      </c>
+      <c r="G1" s="4" t="s">
         <v>106</v>
       </c>
-      <c r="E1" s="4" t="s">
-        <v>107</v>
-      </c>
-      <c r="F1" s="4" t="s">
-        <v>96</v>
-      </c>
-      <c r="G1" s="4" t="s">
-        <v>108</v>
-      </c>
       <c r="H1" s="4" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="I1" s="4" t="s">
         <v>32</v>
@@ -4841,19 +4859,19 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="C1" s="4" t="s">
         <v>65</v>
       </c>
-      <c r="B1" s="4" t="s">
-        <v>66</v>
-      </c>
-      <c r="C1" s="4" t="s">
-        <v>67</v>
-      </c>
       <c r="D1" s="4" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="F1" s="4" t="s">
         <v>32</v>

</xml_diff>